<commit_message>
Refresh 2026-05 release evidence
</commit_message>
<xml_diff>
--- a/output/host_counts_weighted.xlsx
+++ b/output/host_counts_weighted.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="host_counts_weighted" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="host_counts_weighted" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,15 +448,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>王馨</t>
+          <t>徐幻</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3004.68</v>
+        <v>4081</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>王馨 (3004.68)</t>
+          <t>徐幻 (4081.00)</t>
         </is>
       </c>
     </row>
@@ -467,161 +467,101 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2801.05</v>
+        <v>3711</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>孙慧敏 (2801.05)</t>
+          <t>孙慧敏 (3711.00)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>侯翩翩</t>
+          <t>丁俐佳</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2671.68</v>
+        <v>3306</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>侯翩翩 (2671.68)</t>
+          <t>丁俐佳 (3306.00)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>丁俐佳</t>
+          <t>何雯</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2602.05</v>
+        <v>3004</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>丁俐佳 (2602.05)</t>
+          <t>何雯 (3004.00)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>何雯</t>
+          <t>徐欣悦</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2300.55</v>
+        <v>2941</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>何雯 (2300.55)</t>
+          <t>徐欣悦 (2941.00)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>徐幻</t>
+          <t>王馨</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2249.53</v>
+        <v>2707</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>徐幻 (2249.53)</t>
+          <t>王馨 (2707.00)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>徐欣悦</t>
+          <t>侯翩翩</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2014.4</v>
+        <v>2470</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>徐欣悦 (2014.40)</t>
+          <t>侯翩翩 (2470.00)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>桂婕</t>
+          <t>丁汉韬</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>91.75</v>
+        <v>100</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>桂婕 (91.75)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>岳浩然</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>57.25</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>岳浩然 (57.25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>刘花旗</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>48.25</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>刘花旗 (48.25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>王雪</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>44.75</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>王雪 (44.75)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>曹嘉洋</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>曹嘉洋 (3.00)</t>
+          <t>丁汉韬 (100.00)</t>
         </is>
       </c>
     </row>

</xml_diff>